<commit_message>
test(seguimiento): add CE grading example
</commit_message>
<xml_diff>
--- a/SEGUIMIENTO_CURSO_PIA.xlsx
+++ b/SEGUIMIENTO_CURSO_PIA.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Registro_Notas" sheetId="6" r:id="rId6"/>
     <sheet name="RA_CE" sheetId="7" r:id="rId7"/>
     <sheet name="Listas" sheetId="8" r:id="rId8"/>
+    <sheet name="Prueba_CE" sheetId="9" r:id="rId10"/>
   </sheets>
   <calcPr calcMode="auto"/>
 </workbook>
@@ -38380,4 +38381,570 @@
   </sheetData>
   <autoFilter ref="A1:B6"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J16"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="55" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>Alumno</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>Actividad</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>RA</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t>Descripción CE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>Nota CE 0-10</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t>Peso CE %</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t>Nota ponderada CE</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t>Comprobación</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ana Pérez</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1PIA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Titanic EDA</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>RA2</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>RA2.c</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Define el modelo según el problema planteado.</t>
+        </is>
+      </c>
+      <c r="G2">
+        <v>8</v>
+      </c>
+      <c r="H2">
+        <v>60</v>
+      </c>
+      <c r="I2">
+        <f>G2*H2/100</f>
+      </c>
+      <c r="J2">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ana Pérez</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1PIA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Titanic EDA</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>RA2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>RA2.e</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Evalúa los resultados obtenidos.</t>
+        </is>
+      </c>
+      <c r="G3">
+        <v>7</v>
+      </c>
+      <c r="H3">
+        <v>40</v>
+      </c>
+      <c r="I3">
+        <f>G3*H3/100</f>
+      </c>
+      <c r="J3">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bruno Martín</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1PIA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Titanic EDA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>RA2</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>RA2.c</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Define el modelo según el problema planteado.</t>
+        </is>
+      </c>
+      <c r="G4">
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <v>60</v>
+      </c>
+      <c r="I4">
+        <f>G4*H4/100</f>
+      </c>
+      <c r="J4">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Bruno Martín</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1PIA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Titanic EDA</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>RA2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>RA2.e</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Evalúa los resultados obtenidos.</t>
+        </is>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <v>40</v>
+      </c>
+      <c r="I5">
+        <f>G5*H5/100</f>
+      </c>
+      <c r="J5">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ana Pérez</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1PIA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Itinerario R - mini EDA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>RA1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>RA1.d</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Valora características de lenguajes para IA.</t>
+        </is>
+      </c>
+      <c r="G6">
+        <v>9</v>
+      </c>
+      <c r="H6">
+        <v>100</v>
+      </c>
+      <c r="I6">
+        <f>G6*H6/100</f>
+      </c>
+      <c r="J6">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bruno Martín</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1PIA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Itinerario R - mini EDA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>RA1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>RA1.d</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Valora características de lenguajes para IA.</t>
+        </is>
+      </c>
+      <c r="G7">
+        <v>7</v>
+      </c>
+      <c r="H7">
+        <v>100</v>
+      </c>
+      <c r="I7">
+        <f>G7*H7/100</f>
+      </c>
+      <c r="J7">
+        <v>7.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8"/>
+      <c r="B8"/>
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="E8"/>
+      <c r="F8"/>
+      <c r="G8"/>
+      <c r="H8"/>
+      <c r="I8"/>
+      <c r="J8"/>
+    </row>
+    <row r="9">
+      <c r="A9"/>
+      <c r="B9"/>
+      <c r="C9"/>
+      <c r="D9"/>
+      <c r="E9"/>
+      <c r="F9"/>
+      <c r="G9"/>
+      <c r="H9"/>
+      <c r="I9"/>
+      <c r="J9"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="1">
+        <is>
+          <t>Alumno</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="1">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="1">
+        <is>
+          <t>Media CE</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="1">
+        <is>
+          <t>Suma ponderada CE</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="1">
+        <is>
+          <t>Actividades/CE</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="1">
+        <is>
+          <t>Pendientes esperados</t>
+        </is>
+      </c>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ana Pérez</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>RA2.c</t>
+        </is>
+      </c>
+      <c r="C11">
+        <f>AVERAGEIFS($G$2:$G$7,$A$2:$A$7,A11,$E$2:$E$7,B11)</f>
+      </c>
+      <c r="D11">
+        <f>SUMIFS($I$2:$I$7,$A$2:$A$7,A11,$E$2:$E$7,B11)</f>
+      </c>
+      <c r="E11">
+        <f>COUNTIFS($A$2:$A$7,A11,$E$2:$E$7,B11)</f>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11"/>
+      <c r="H11"/>
+      <c r="I11"/>
+      <c r="J11"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ana Pérez</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>RA2.e</t>
+        </is>
+      </c>
+      <c r="C12">
+        <f>AVERAGEIFS($G$2:$G$7,$A$2:$A$7,A12,$E$2:$E$7,B12)</f>
+      </c>
+      <c r="D12">
+        <f>SUMIFS($I$2:$I$7,$A$2:$A$7,A12,$E$2:$E$7,B12)</f>
+      </c>
+      <c r="E12">
+        <f>COUNTIFS($A$2:$A$7,A12,$E$2:$E$7,B12)</f>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12"/>
+      <c r="H12"/>
+      <c r="I12"/>
+      <c r="J12"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Ana Pérez</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RA1.d</t>
+        </is>
+      </c>
+      <c r="C13">
+        <f>AVERAGEIFS($G$2:$G$7,$A$2:$A$7,A13,$E$2:$E$7,B13)</f>
+      </c>
+      <c r="D13">
+        <f>SUMIFS($I$2:$I$7,$A$2:$A$7,A13,$E$2:$E$7,B13)</f>
+      </c>
+      <c r="E13">
+        <f>COUNTIFS($A$2:$A$7,A13,$E$2:$E$7,B13)</f>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13"/>
+      <c r="H13"/>
+      <c r="I13"/>
+      <c r="J13"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Bruno Martín</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>RA2.c</t>
+        </is>
+      </c>
+      <c r="C14">
+        <f>AVERAGEIFS($G$2:$G$7,$A$2:$A$7,A14,$E$2:$E$7,B14)</f>
+      </c>
+      <c r="D14">
+        <f>SUMIFS($I$2:$I$7,$A$2:$A$7,A14,$E$2:$E$7,B14)</f>
+      </c>
+      <c r="E14">
+        <f>COUNTIFS($A$2:$A$7,A14,$E$2:$E$7,B14)</f>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14"/>
+      <c r="H14"/>
+      <c r="I14"/>
+      <c r="J14"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Bruno Martín</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>RA2.e</t>
+        </is>
+      </c>
+      <c r="C15">
+        <f>AVERAGEIFS($G$2:$G$7,$A$2:$A$7,A15,$E$2:$E$7,B15)</f>
+      </c>
+      <c r="D15">
+        <f>SUMIFS($I$2:$I$7,$A$2:$A$7,A15,$E$2:$E$7,B15)</f>
+      </c>
+      <c r="E15">
+        <f>COUNTIFS($A$2:$A$7,A15,$E$2:$E$7,B15)</f>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15"/>
+      <c r="H15"/>
+      <c r="I15"/>
+      <c r="J15"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Bruno Martín</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>RA1.d</t>
+        </is>
+      </c>
+      <c r="C16">
+        <f>AVERAGEIFS($G$2:$G$7,$A$2:$A$7,A16,$E$2:$E$7,B16)</f>
+      </c>
+      <c r="D16">
+        <f>SUMIFS($I$2:$I$7,$A$2:$A$7,A16,$E$2:$E$7,B16)</f>
+      </c>
+      <c r="E16">
+        <f>COUNTIFS($A$2:$A$7,A16,$E$2:$E$7,B16)</f>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16"/>
+      <c r="H16"/>
+      <c r="I16"/>
+      <c r="J16"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J8"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(ud1): add language and format comparison evidence
</commit_message>
<xml_diff>
--- a/SEGUIMIENTO_CURSO_PIA.xlsx
+++ b/SEGUIMIENTO_CURSO_PIA.xlsx
@@ -3421,7 +3421,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P280"/>
+  <dimension ref="A1:P281"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -16916,8 +16916,64 @@
       <c r="O280"/>
       <c r="P280"/>
     </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>01 - Fundamentos de Python</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Actividad breve — Comparativa de lenguajes y formatos para IA</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>guía/rúbrica</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>01-fundamentos-python/04-evaluacion/comparativa-lenguajes-formatos-ia.md</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>RA1.b; RA1.c; RA1.d; RA1.e; RA1.f</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I281"/>
+      <c r="J281"/>
+      <c r="K281"/>
+      <c r="L281"/>
+      <c r="M281">
+        <f>IF(AND(ISNUMBER(K281),ISNUMBER(L281)),MAX(K281-L281,0),"")</f>
+      </c>
+      <c r="N281"/>
+      <c r="O281"/>
+      <c r="P281" t="inlineStr">
+        <is>
+          <t>Evidencia formal RD 279/2021 para idoneidad de lenguajes y formatos/marcado.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P280"/>
+  <autoFilter ref="A1:P281"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F1000">
       <formula1>"Sí,No,Revisar"</formula1>

</xml_diff>